<commit_message>
inplementing some MS comparisons and searches in Jupyter notebook
</commit_message>
<xml_diff>
--- a/src/Humancheck_revised_zfNGbrain_20221129_1219_proc3_noques_noNa.xlsx
+++ b/src/Humancheck_revised_zfNGbrain_20221129_1219_proc3_noques_noNa.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\其他電腦\My Computer\GlycoMSParser\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72008E2C-DA7C-4809-B4CD-3BBB7407CA47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E3BF488-E977-4F2B-82FA-944F96A83E5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6255" yWindow="2025" windowWidth="21600" windowHeight="13515" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12645" yWindow="810" windowWidth="14730" windowHeight="13515" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="revised_zfNGbrain_20221129_1219" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1071" uniqueCount="582">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1071" uniqueCount="583">
   <si>
     <t>MS1scan no</t>
   </si>
@@ -1798,6 +1798,10 @@
   </si>
   <si>
     <t>12 bisecting</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>F1H5N4S1</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
@@ -3003,6 +3007,9 @@
   <sheetPr filterMode="1"/>
   <dimension ref="A1:XFD259"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="20.875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:23 16384:16384" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -5717,7 +5724,7 @@
         <v>2583.3168000000001</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>53</v>
+        <v>582</v>
       </c>
       <c r="E39" t="s">
         <v>54</v>
@@ -7852,7 +7859,7 @@
       <c r="E69" t="s">
         <v>197</v>
       </c>
-      <c r="F69">
+      <c r="F69" s="3">
         <v>22567</v>
       </c>
       <c r="G69" t="s">

</xml_diff>